<commit_message>
manually calculated SSE, RMSE, SST, R Square in excel sheet
</commit_message>
<xml_diff>
--- a/Motor_Insurance_Regression/ClaimsVsPayment.xlsx
+++ b/Motor_Insurance_Regression/ClaimsVsPayment.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
   <si>
     <t>X(independent)</t>
   </si>
@@ -45,15 +45,6 @@
     <t>avg of Y values</t>
   </si>
   <si>
-    <t>Y^ (Predcited)</t>
-  </si>
-  <si>
-    <t>y-y^</t>
-  </si>
-  <si>
-    <t>(y-y^)sqre</t>
-  </si>
-  <si>
     <t>SSE</t>
   </si>
   <si>
@@ -61,6 +52,24 @@
   </si>
   <si>
     <t>R^2</t>
+  </si>
+  <si>
+    <t>yi-y^</t>
+  </si>
+  <si>
+    <t>(yi-y^)sqre</t>
+  </si>
+  <si>
+    <t>yi-mean(y)</t>
+  </si>
+  <si>
+    <t>(yi-mean(y))sqre</t>
+  </si>
+  <si>
+    <t>Y^ (Predicted)</t>
+  </si>
+  <si>
+    <t>explained variation/total variation</t>
   </si>
 </sst>
 </file>
@@ -114,9 +123,7 @@
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:chart>
-    <c:title>
-      <c:layout/>
-    </c:title>
+    <c:title/>
     <c:plotArea>
       <c:layout/>
       <c:scatterChart>
@@ -144,7 +151,6 @@
             <c:trendlineType val="linear"/>
             <c:dispEq val="1"/>
             <c:trendlineLbl>
-              <c:layout/>
               <c:numFmt formatCode="General" sourceLinked="0"/>
             </c:trendlineLbl>
           </c:trendline>
@@ -545,23 +551,23 @@
             </c:numRef>
           </c:yVal>
         </c:ser>
-        <c:axId val="84553088"/>
-        <c:axId val="84554880"/>
+        <c:axId val="67628416"/>
+        <c:axId val="67708032"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="84553088"/>
+        <c:axId val="67628416"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="b"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="84554880"/>
+        <c:crossAx val="67708032"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="84554880"/>
+        <c:axId val="67708032"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -569,20 +575,19 @@
         <c:majorGridlines/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="84553088"/>
+        <c:crossAx val="67628416"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
-      <c:layout/>
     </c:legend>
     <c:plotVisOnly val="1"/>
   </c:chart>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75000000000000022" l="0.70000000000000018" r="0.70000000000000018" t="0.75000000000000022" header="0.3000000000000001" footer="0.3000000000000001"/>
+    <c:pageMargins b="0.75000000000000033" l="0.70000000000000029" r="0.70000000000000029" t="0.75000000000000033" header="0.30000000000000016" footer="0.30000000000000016"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -720,23 +725,23 @@
             </c:numRef>
           </c:yVal>
         </c:ser>
-        <c:axId val="82578048"/>
-        <c:axId val="82579840"/>
+        <c:axId val="67758720"/>
+        <c:axId val="67895680"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="82578048"/>
+        <c:axId val="67758720"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="b"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="82579840"/>
+        <c:crossAx val="67895680"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="82579840"/>
+        <c:axId val="67895680"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -744,7 +749,7 @@
         <c:majorGridlines/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="82578048"/>
+        <c:crossAx val="67758720"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -757,7 +762,7 @@
   </c:chart>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75000000000000022" l="0.70000000000000018" r="0.70000000000000018" t="0.75000000000000022" header="0.3000000000000001" footer="0.3000000000000001"/>
+    <c:pageMargins b="0.75000000000000033" l="0.70000000000000029" r="0.70000000000000029" t="0.75000000000000033" header="0.30000000000000016" footer="0.30000000000000016"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -830,23 +835,23 @@
             </c:numRef>
           </c:yVal>
         </c:ser>
-        <c:axId val="13480320"/>
-        <c:axId val="57461376"/>
+        <c:axId val="67948928"/>
+        <c:axId val="67950464"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="13480320"/>
+        <c:axId val="67948928"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="b"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="57461376"/>
+        <c:crossAx val="67950464"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="57461376"/>
+        <c:axId val="67950464"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -854,7 +859,7 @@
         <c:majorGridlines/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="13480320"/>
+        <c:crossAx val="67948928"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -867,7 +872,7 @@
   </c:chart>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageMargins b="0.75000000000000011" l="0.70000000000000007" r="0.70000000000000007" t="0.75000000000000011" header="0.30000000000000004" footer="0.30000000000000004"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -947,16 +952,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>419100</xdr:colOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>352425</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>66675</xdr:rowOff>
+      <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
       <xdr:row>20</xdr:row>
-      <xdr:rowOff>142875</xdr:rowOff>
+      <xdr:rowOff>171450</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1911,15 +1916,17 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="4" max="4" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="32.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -1933,23 +1940,29 @@
         <v>7</v>
       </c>
       <c r="E1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="F1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
+        <v>13</v>
+      </c>
+      <c r="H1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="D2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:9">
       <c r="A3" s="1">
         <v>0</v>
       </c>
@@ -1972,8 +1985,16 @@
         <f>F3^2</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:7">
+      <c r="H3">
+        <f>B3-$D$3</f>
+        <v>-2</v>
+      </c>
+      <c r="I3">
+        <f>H3^2</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
       <c r="A4" s="1">
         <v>1</v>
       </c>
@@ -1992,8 +2013,16 @@
         <f t="shared" ref="G4:G5" si="2">F4^2</f>
         <v>9</v>
       </c>
-    </row>
-    <row r="5" spans="1:7">
+      <c r="H4">
+        <f t="shared" ref="H4:H5" si="3">B4-$D$3</f>
+        <v>-2</v>
+      </c>
+      <c r="I4">
+        <f t="shared" ref="I4:I5" si="4">H4^2</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
       <c r="A5" s="1">
         <v>1</v>
       </c>
@@ -2012,49 +2041,71 @@
         <f t="shared" si="2"/>
         <v>9</v>
       </c>
-    </row>
-    <row r="6" spans="1:7">
+      <c r="H5">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="I5">
+        <f t="shared" si="4"/>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:9">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="D7" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7">
+        <v>9</v>
+      </c>
+      <c r="G7">
         <f>SUM(G3:G5)</f>
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:9">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="D8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
+        <v>10</v>
+      </c>
+      <c r="I8">
+        <f>SUM(I3:I5)</f>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="D9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
+        <v>11</v>
+      </c>
+      <c r="F9">
+        <f>1-(G7/I8)</f>
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:9">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
-    </row>
-    <row r="12" spans="1:7">
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:9">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
     </row>

</xml_diff>

<commit_message>
Added code to plot simple regression model - one variable
</commit_message>
<xml_diff>
--- a/Motor_Insurance_Regression/ClaimsVsPayment.xlsx
+++ b/Motor_Insurance_Regression/ClaimsVsPayment.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="75" windowWidth="20055" windowHeight="7935" activeTab="2"/>
+    <workbookView xWindow="240" yWindow="75" windowWidth="20055" windowHeight="7935" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="ClaimsVsPayment" sheetId="1" r:id="rId1"/>
@@ -22,12 +22,6 @@
   </si>
   <si>
     <t>Y(dependent)</t>
-  </si>
-  <si>
-    <t>X(independent)-number of claims</t>
-  </si>
-  <si>
-    <t>Y(dependent)-total payment for all the claims</t>
   </si>
   <si>
     <t>Xi</t>
@@ -70,6 +64,12 @@
   </si>
   <si>
     <t>explained variation/total variation</t>
+  </si>
+  <si>
+    <t>payment</t>
+  </si>
+  <si>
+    <t>claims</t>
   </si>
 </sst>
 </file>
@@ -551,23 +551,23 @@
             </c:numRef>
           </c:yVal>
         </c:ser>
-        <c:axId val="67628416"/>
-        <c:axId val="67708032"/>
+        <c:axId val="88681856"/>
+        <c:axId val="88695936"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="67628416"/>
+        <c:axId val="88681856"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="b"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="67708032"/>
+        <c:crossAx val="88695936"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="67708032"/>
+        <c:axId val="88695936"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -575,7 +575,7 @@
         <c:majorGridlines/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="67628416"/>
+        <c:crossAx val="88681856"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -587,7 +587,7 @@
   </c:chart>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75000000000000033" l="0.70000000000000029" r="0.70000000000000029" t="0.75000000000000033" header="0.30000000000000016" footer="0.30000000000000016"/>
+    <c:pageMargins b="0.75000000000000044" l="0.7000000000000004" r="0.7000000000000004" t="0.75000000000000044" header="0.30000000000000021" footer="0.30000000000000021"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -613,7 +613,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Y(dependent)-total payment for all the claims</c:v>
+                  <c:v>payment</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -725,23 +725,23 @@
             </c:numRef>
           </c:yVal>
         </c:ser>
-        <c:axId val="67758720"/>
-        <c:axId val="67895680"/>
+        <c:axId val="71404160"/>
+        <c:axId val="71405952"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="67758720"/>
+        <c:axId val="71404160"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="b"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="67895680"/>
+        <c:crossAx val="71405952"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="67895680"/>
+        <c:axId val="71405952"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -749,7 +749,7 @@
         <c:majorGridlines/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="67758720"/>
+        <c:crossAx val="71404160"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -762,7 +762,7 @@
   </c:chart>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75000000000000033" l="0.70000000000000029" r="0.70000000000000029" t="0.75000000000000033" header="0.30000000000000016" footer="0.30000000000000016"/>
+    <c:pageMargins b="0.75000000000000044" l="0.7000000000000004" r="0.7000000000000004" t="0.75000000000000044" header="0.30000000000000021" footer="0.30000000000000021"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -835,23 +835,23 @@
             </c:numRef>
           </c:yVal>
         </c:ser>
-        <c:axId val="67948928"/>
-        <c:axId val="67950464"/>
+        <c:axId val="71430528"/>
+        <c:axId val="71432064"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="67948928"/>
+        <c:axId val="71430528"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="b"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="67950464"/>
+        <c:crossAx val="71432064"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="67950464"/>
+        <c:axId val="71432064"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -859,7 +859,7 @@
         <c:majorGridlines/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="67948928"/>
+        <c:crossAx val="71430528"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -872,7 +872,7 @@
   </c:chart>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75000000000000011" l="0.70000000000000007" r="0.70000000000000007" t="0.75000000000000011" header="0.30000000000000004" footer="0.30000000000000004"/>
+    <c:pageMargins b="0.75000000000000022" l="0.70000000000000018" r="0.70000000000000018" t="0.75000000000000022" header="0.3000000000000001" footer="0.3000000000000001"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -1806,10 +1806,10 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>3</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -1928,38 +1928,38 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" t="s">
         <v>5</v>
       </c>
-      <c r="C1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D1" t="s">
-        <v>7</v>
-      </c>
       <c r="E1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" t="s">
         <v>12</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>13</v>
-      </c>
-      <c r="H1" t="s">
-        <v>14</v>
-      </c>
-      <c r="I1" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="D2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -2058,7 +2058,7 @@
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="D7" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G7">
         <f>SUM(G3:G5)</f>
@@ -2069,7 +2069,7 @@
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="D8" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="I8">
         <f>SUM(I3:I5)</f>
@@ -2080,7 +2080,7 @@
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="D9" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F9">
         <f>1-(G7/I8)</f>
@@ -2095,10 +2095,10 @@
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="D11" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E11" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:9">

</xml_diff>

<commit_message>
Added code to calculate SSE
</commit_message>
<xml_diff>
--- a/Motor_Insurance_Regression/ClaimsVsPayment.xlsx
+++ b/Motor_Insurance_Regression/ClaimsVsPayment.xlsx
@@ -84,12 +84,6 @@
     <t>error square</t>
   </si>
   <si>
-    <t>slope</t>
-  </si>
-  <si>
-    <t>intercept</t>
-  </si>
-  <si>
     <t>y - predicted</t>
   </si>
   <si>
@@ -106,6 +100,12 @@
   </si>
   <si>
     <t>Y</t>
+  </si>
+  <si>
+    <t>y=3.413x+19.99</t>
+  </si>
+  <si>
+    <t>sse</t>
   </si>
 </sst>
 </file>
@@ -590,23 +590,23 @@
             </c:numRef>
           </c:yVal>
         </c:ser>
-        <c:axId val="74136960"/>
-        <c:axId val="74151040"/>
+        <c:axId val="68107648"/>
+        <c:axId val="68121728"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="74136960"/>
+        <c:axId val="68107648"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="b"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="74151040"/>
+        <c:crossAx val="68121728"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="74151040"/>
+        <c:axId val="68121728"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -614,7 +614,7 @@
         <c:majorGridlines/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="74136960"/>
+        <c:crossAx val="68107648"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -627,7 +627,7 @@
   </c:chart>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75000000000000078" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000078" header="0.30000000000000032" footer="0.30000000000000032"/>
+    <c:pageMargins b="0.75000000000000089" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000089" header="0.30000000000000032" footer="0.30000000000000032"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -768,23 +768,23 @@
             </c:numRef>
           </c:yVal>
         </c:ser>
-        <c:axId val="81968512"/>
-        <c:axId val="81970304"/>
+        <c:axId val="80653696"/>
+        <c:axId val="80655488"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="81968512"/>
+        <c:axId val="80653696"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="b"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="81970304"/>
+        <c:crossAx val="80655488"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="81970304"/>
+        <c:axId val="80655488"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -792,7 +792,7 @@
         <c:majorGridlines/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="81968512"/>
+        <c:crossAx val="80653696"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -805,7 +805,7 @@
   </c:chart>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75000000000000078" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000078" header="0.30000000000000032" footer="0.30000000000000032"/>
+    <c:pageMargins b="0.75000000000000089" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000089" header="0.30000000000000032" footer="0.30000000000000032"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -878,23 +878,23 @@
             </c:numRef>
           </c:yVal>
         </c:ser>
-        <c:axId val="81978496"/>
-        <c:axId val="81980032"/>
+        <c:axId val="80667776"/>
+        <c:axId val="80669312"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="81978496"/>
+        <c:axId val="80667776"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="b"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="81980032"/>
+        <c:crossAx val="80669312"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="81980032"/>
+        <c:axId val="80669312"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -902,7 +902,7 @@
         <c:majorGridlines/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="81978496"/>
+        <c:crossAx val="80667776"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -915,7 +915,7 @@
   </c:chart>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75000000000000044" l="0.7000000000000004" r="0.7000000000000004" t="0.75000000000000044" header="0.30000000000000021" footer="0.30000000000000021"/>
+    <c:pageMargins b="0.75000000000000056" l="0.70000000000000051" r="0.70000000000000051" t="0.75000000000000056" header="0.30000000000000027" footer="0.30000000000000027"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -925,13 +925,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>11</xdr:col>
+      <xdr:col>10</xdr:col>
       <xdr:colOff>485775</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
+      <xdr:col>18</xdr:col>
       <xdr:colOff>180975</xdr:colOff>
       <xdr:row>20</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -1318,17 +1318,18 @@
     <col min="2" max="2" width="14.28515625" customWidth="1"/>
     <col min="4" max="4" width="15.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.85546875" customWidth="1"/>
-    <col min="9" max="9" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C1" t="s">
         <v>19</v>
@@ -1340,22 +1341,22 @@
         <v>21</v>
       </c>
       <c r="F1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
-        <v>25</v>
-      </c>
       <c r="K1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:11">
@@ -1381,6 +1382,22 @@
         <f>SUM(E2:E64)</f>
         <v>472818.28984126967</v>
       </c>
+      <c r="H2">
+        <f>(3.413*A2)+19.99</f>
+        <v>388.59399999999999</v>
+      </c>
+      <c r="I2">
+        <f>B2-H2</f>
+        <v>3.9060000000000059</v>
+      </c>
+      <c r="J2">
+        <f>I2*I2</f>
+        <v>15.256836000000046</v>
+      </c>
+      <c r="K2">
+        <f>SUM(J2:J64)</f>
+        <v>78796.798828999992</v>
+      </c>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="1">
@@ -1397,6 +1414,18 @@
         <f t="shared" ref="E3:E64" si="1">D3*D3</f>
         <v>2702.6795263290501</v>
       </c>
+      <c r="H3">
+        <f t="shared" ref="H3:H64" si="2">(3.413*A3)+19.99</f>
+        <v>84.836999999999989</v>
+      </c>
+      <c r="I3">
+        <f t="shared" ref="I3:I64" si="3">B3-H3</f>
+        <v>-38.636999999999986</v>
+      </c>
+      <c r="J3">
+        <f t="shared" ref="J3:J64" si="4">I3*I3</f>
+        <v>1492.8177689999989</v>
+      </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" s="1">
@@ -1413,6 +1442,18 @@
         <f t="shared" si="1"/>
         <v>6804.1549231544468</v>
       </c>
+      <c r="H4">
+        <f t="shared" si="2"/>
+        <v>64.358999999999995</v>
+      </c>
+      <c r="I4">
+        <f t="shared" si="3"/>
+        <v>-48.658999999999992</v>
+      </c>
+      <c r="J4">
+        <f t="shared" si="4"/>
+        <v>2367.698280999999</v>
+      </c>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" s="1">
@@ -1429,6 +1470,18 @@
         <f t="shared" si="1"/>
         <v>104984.22873267825</v>
       </c>
+      <c r="H5">
+        <f t="shared" si="2"/>
+        <v>443.202</v>
+      </c>
+      <c r="I5">
+        <f t="shared" si="3"/>
+        <v>-21.00200000000001</v>
+      </c>
+      <c r="J5">
+        <f t="shared" si="4"/>
+        <v>441.08400400000039</v>
+      </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="1">
@@ -1445,6 +1498,18 @@
         <f t="shared" si="1"/>
         <v>449.9785739480979</v>
       </c>
+      <c r="H6">
+        <f t="shared" si="2"/>
+        <v>156.51</v>
+      </c>
+      <c r="I6">
+        <f t="shared" si="3"/>
+        <v>-37.109999999999985</v>
+      </c>
+      <c r="J6">
+        <f t="shared" si="4"/>
+        <v>1377.1520999999989</v>
+      </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="1">
@@ -1461,6 +1526,18 @@
         <f t="shared" si="1"/>
         <v>5287.1365104560346</v>
       </c>
+      <c r="H7">
+        <f t="shared" si="2"/>
+        <v>214.53100000000001</v>
+      </c>
+      <c r="I7">
+        <f t="shared" si="3"/>
+        <v>-43.631</v>
+      </c>
+      <c r="J7">
+        <f t="shared" si="4"/>
+        <v>1903.6641609999999</v>
+      </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="1">
@@ -1477,6 +1554,18 @@
         <f t="shared" si="1"/>
         <v>1704.6412723607966</v>
       </c>
+      <c r="H8">
+        <f t="shared" si="2"/>
+        <v>98.48899999999999</v>
+      </c>
+      <c r="I8">
+        <f t="shared" si="3"/>
+        <v>-41.588999999999992</v>
+      </c>
+      <c r="J8">
+        <f t="shared" si="4"/>
+        <v>1729.6449209999994</v>
+      </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" s="1">
@@ -1493,6 +1582,18 @@
         <f t="shared" si="1"/>
         <v>427.96444696397089</v>
       </c>
+      <c r="H9">
+        <f t="shared" si="2"/>
+        <v>67.771999999999991</v>
+      </c>
+      <c r="I9">
+        <f t="shared" si="3"/>
+        <v>9.7280000000000086</v>
+      </c>
+      <c r="J9">
+        <f t="shared" si="4"/>
+        <v>94.633984000000169</v>
+      </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="1">
@@ -1509,6 +1610,18 @@
         <f t="shared" si="1"/>
         <v>13412.581113630637</v>
       </c>
+      <c r="H10">
+        <f t="shared" si="2"/>
+        <v>173.57499999999999</v>
+      </c>
+      <c r="I10">
+        <f t="shared" si="3"/>
+        <v>40.425000000000011</v>
+      </c>
+      <c r="J10">
+        <f t="shared" si="4"/>
+        <v>1634.1806250000009</v>
+      </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" s="1">
@@ -1525,6 +1638,18 @@
         <f t="shared" si="1"/>
         <v>1081.5746056941298</v>
       </c>
+      <c r="H11">
+        <f t="shared" si="2"/>
+        <v>54.11999999999999</v>
+      </c>
+      <c r="I11">
+        <f t="shared" si="3"/>
+        <v>11.180000000000007</v>
+      </c>
+      <c r="J11">
+        <f t="shared" si="4"/>
+        <v>124.99240000000015</v>
+      </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" s="1">
@@ -1541,6 +1666,18 @@
         <f t="shared" si="1"/>
         <v>5973.3269866465098</v>
       </c>
+      <c r="H12">
+        <f t="shared" si="2"/>
+        <v>37.054999999999993</v>
+      </c>
+      <c r="I12">
+        <f t="shared" si="3"/>
+        <v>-16.154999999999994</v>
+      </c>
+      <c r="J12">
+        <f t="shared" si="4"/>
+        <v>260.9840249999998</v>
+      </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" s="1">
@@ -1557,6 +1694,18 @@
         <f t="shared" si="1"/>
         <v>22473.817145376666</v>
       </c>
+      <c r="H13">
+        <f t="shared" si="2"/>
+        <v>183.81399999999999</v>
+      </c>
+      <c r="I13">
+        <f t="shared" si="3"/>
+        <v>64.286000000000001</v>
+      </c>
+      <c r="J13">
+        <f t="shared" si="4"/>
+        <v>4132.6897960000006</v>
+      </c>
     </row>
     <row r="14" spans="1:11">
       <c r="A14" s="1">
@@ -1573,6 +1722,18 @@
         <f t="shared" si="1"/>
         <v>5578.1930183925424</v>
       </c>
+      <c r="H14">
+        <f t="shared" si="2"/>
+        <v>57.533000000000001</v>
+      </c>
+      <c r="I14">
+        <f t="shared" si="3"/>
+        <v>-34.033000000000001</v>
+      </c>
+      <c r="J14">
+        <f t="shared" si="4"/>
+        <v>1158.245089</v>
+      </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" s="1">
@@ -1589,6 +1750,18 @@
         <f t="shared" si="1"/>
         <v>3432.4719072814314</v>
       </c>
+      <c r="H15">
+        <f t="shared" si="2"/>
+        <v>98.48899999999999</v>
+      </c>
+      <c r="I15">
+        <f t="shared" si="3"/>
+        <v>-58.888999999999989</v>
+      </c>
+      <c r="J15">
+        <f t="shared" si="4"/>
+        <v>3467.9143209999988</v>
+      </c>
     </row>
     <row r="16" spans="1:11">
       <c r="A16" s="1">
@@ -1605,8 +1778,20 @@
         <f t="shared" si="1"/>
         <v>2439.1055580750826</v>
       </c>
-    </row>
-    <row r="17" spans="1:5">
+      <c r="H16">
+        <f t="shared" si="2"/>
+        <v>43.881</v>
+      </c>
+      <c r="I16">
+        <f t="shared" si="3"/>
+        <v>4.9189999999999969</v>
+      </c>
+      <c r="J16">
+        <f t="shared" si="4"/>
+        <v>24.196560999999971</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10">
       <c r="A17" s="1">
         <v>2</v>
       </c>
@@ -1621,8 +1806,20 @@
         <f t="shared" si="1"/>
         <v>8388.2338120433378</v>
       </c>
-    </row>
-    <row r="18" spans="1:5">
+      <c r="H17">
+        <f t="shared" si="2"/>
+        <v>26.815999999999999</v>
+      </c>
+      <c r="I17">
+        <f t="shared" si="3"/>
+        <v>-20.216000000000001</v>
+      </c>
+      <c r="J17">
+        <f t="shared" si="4"/>
+        <v>408.68665600000003</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10">
       <c r="A18" s="1">
         <v>24</v>
       </c>
@@ -1637,8 +1834,20 @@
         <f t="shared" si="1"/>
         <v>1347.8222247417489</v>
       </c>
-    </row>
-    <row r="19" spans="1:5">
+      <c r="H18">
+        <f t="shared" si="2"/>
+        <v>101.90199999999999</v>
+      </c>
+      <c r="I18">
+        <f t="shared" si="3"/>
+        <v>32.998000000000019</v>
+      </c>
+      <c r="J18">
+        <f t="shared" si="4"/>
+        <v>1088.8680040000013</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10">
       <c r="A19" s="1">
         <v>6</v>
       </c>
@@ -1653,8 +1862,20 @@
         <f t="shared" si="1"/>
         <v>2236.0888914084157</v>
       </c>
-    </row>
-    <row r="20" spans="1:5">
+      <c r="H19">
+        <f t="shared" si="2"/>
+        <v>40.467999999999996</v>
+      </c>
+      <c r="I19">
+        <f t="shared" si="3"/>
+        <v>10.432000000000002</v>
+      </c>
+      <c r="J19">
+        <f t="shared" si="4"/>
+        <v>108.82662400000004</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10">
       <c r="A20" s="1">
         <v>3</v>
       </c>
@@ -1669,8 +1890,20 @@
         <f t="shared" si="1"/>
         <v>8796.0579390274615</v>
       </c>
-    </row>
-    <row r="21" spans="1:5">
+      <c r="H20">
+        <f t="shared" si="2"/>
+        <v>30.228999999999999</v>
+      </c>
+      <c r="I20">
+        <f t="shared" si="3"/>
+        <v>-25.829000000000001</v>
+      </c>
+      <c r="J20">
+        <f t="shared" si="4"/>
+        <v>667.13724100000002</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10">
       <c r="A21" s="1">
         <v>23</v>
       </c>
@@ -1685,8 +1918,20 @@
         <f t="shared" si="1"/>
         <v>219.41603426555798</v>
       </c>
-    </row>
-    <row r="22" spans="1:5">
+      <c r="H21">
+        <f t="shared" si="2"/>
+        <v>98.48899999999999</v>
+      </c>
+      <c r="I21">
+        <f t="shared" si="3"/>
+        <v>14.51100000000001</v>
+      </c>
+      <c r="J21">
+        <f t="shared" si="4"/>
+        <v>210.56912100000028</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10">
       <c r="A22" s="1">
         <v>6</v>
       </c>
@@ -1701,8 +1946,20 @@
         <f t="shared" si="1"/>
         <v>6953.4420660115911</v>
       </c>
-    </row>
-    <row r="23" spans="1:5">
+      <c r="H22">
+        <f t="shared" si="2"/>
+        <v>40.467999999999996</v>
+      </c>
+      <c r="I22">
+        <f t="shared" si="3"/>
+        <v>-25.667999999999996</v>
+      </c>
+      <c r="J22">
+        <f t="shared" si="4"/>
+        <v>658.84622399999978</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10">
       <c r="A23" s="1">
         <v>9</v>
       </c>
@@ -1717,8 +1974,20 @@
         <f t="shared" si="1"/>
         <v>2448.9930183925421</v>
       </c>
-    </row>
-    <row r="24" spans="1:5">
+      <c r="H23">
+        <f t="shared" si="2"/>
+        <v>50.706999999999994</v>
+      </c>
+      <c r="I23">
+        <f t="shared" si="3"/>
+        <v>-2.0069999999999908</v>
+      </c>
+      <c r="J23">
+        <f t="shared" si="4"/>
+        <v>4.0280489999999629</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10">
       <c r="A24" s="1">
         <v>9</v>
       </c>
@@ -1733,8 +2002,20 @@
         <f t="shared" si="1"/>
         <v>2124.0393675988917</v>
       </c>
-    </row>
-    <row r="25" spans="1:5">
+      <c r="H24">
+        <f t="shared" si="2"/>
+        <v>50.706999999999994</v>
+      </c>
+      <c r="I24">
+        <f t="shared" si="3"/>
+        <v>1.3930000000000078</v>
+      </c>
+      <c r="J24">
+        <f t="shared" si="4"/>
+        <v>1.9404490000000216</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10">
       <c r="A25" s="1">
         <v>3</v>
       </c>
@@ -1749,8 +2030,20 @@
         <f t="shared" si="1"/>
         <v>7222.8414310909548</v>
       </c>
-    </row>
-    <row r="26" spans="1:5">
+      <c r="H25">
+        <f t="shared" si="2"/>
+        <v>30.228999999999999</v>
+      </c>
+      <c r="I25">
+        <f t="shared" si="3"/>
+        <v>-17.029</v>
+      </c>
+      <c r="J25">
+        <f t="shared" si="4"/>
+        <v>289.98684099999997</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10">
       <c r="A26" s="1">
         <v>29</v>
       </c>
@@ -1765,8 +2058,20 @@
         <f t="shared" si="1"/>
         <v>32.634923154446994</v>
       </c>
-    </row>
-    <row r="27" spans="1:5">
+      <c r="H26">
+        <f t="shared" si="2"/>
+        <v>118.96699999999998</v>
+      </c>
+      <c r="I26">
+        <f t="shared" si="3"/>
+        <v>-15.066999999999979</v>
+      </c>
+      <c r="J26">
+        <f t="shared" si="4"/>
+        <v>227.01448899999937</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10">
       <c r="A27" s="1">
         <v>7</v>
       </c>
@@ -1781,8 +2086,20 @@
         <f t="shared" si="1"/>
         <v>427.96444696397089</v>
       </c>
-    </row>
-    <row r="28" spans="1:5">
+      <c r="H27">
+        <f t="shared" si="2"/>
+        <v>43.881</v>
+      </c>
+      <c r="I27">
+        <f t="shared" si="3"/>
+        <v>33.619</v>
+      </c>
+      <c r="J27">
+        <f t="shared" si="4"/>
+        <v>1130.237161</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10">
       <c r="A28" s="1">
         <v>4</v>
       </c>
@@ -1797,8 +2114,20 @@
         <f t="shared" si="1"/>
         <v>7462.7658755354005</v>
       </c>
-    </row>
-    <row r="29" spans="1:5">
+      <c r="H28">
+        <f t="shared" si="2"/>
+        <v>33.641999999999996</v>
+      </c>
+      <c r="I28">
+        <f t="shared" si="3"/>
+        <v>-21.841999999999995</v>
+      </c>
+      <c r="J28">
+        <f t="shared" si="4"/>
+        <v>477.07296399999979</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10">
       <c r="A29" s="1">
         <v>20</v>
       </c>
@@ -1813,8 +2142,20 @@
         <f t="shared" si="1"/>
         <v>7.6215671453781662E-3</v>
       </c>
-    </row>
-    <row r="30" spans="1:5">
+      <c r="H29">
+        <f t="shared" si="2"/>
+        <v>88.249999999999986</v>
+      </c>
+      <c r="I29">
+        <f t="shared" si="3"/>
+        <v>9.8500000000000085</v>
+      </c>
+      <c r="J29">
+        <f t="shared" si="4"/>
+        <v>97.022500000000164</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10">
       <c r="A30" s="1">
         <v>7</v>
       </c>
@@ -1829,8 +2170,20 @@
         <f t="shared" si="1"/>
         <v>4940.3047644242879</v>
       </c>
-    </row>
-    <row r="31" spans="1:5">
+      <c r="H30">
+        <f t="shared" si="2"/>
+        <v>43.881</v>
+      </c>
+      <c r="I30">
+        <f t="shared" si="3"/>
+        <v>-15.981000000000002</v>
+      </c>
+      <c r="J30">
+        <f t="shared" si="4"/>
+        <v>255.39236100000005</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10">
       <c r="A31" s="1">
         <v>4</v>
       </c>
@@ -1845,8 +2198,20 @@
         <f t="shared" si="1"/>
         <v>3610.483812043336</v>
       </c>
-    </row>
-    <row r="32" spans="1:5">
+      <c r="H31">
+        <f t="shared" si="2"/>
+        <v>33.641999999999996</v>
+      </c>
+      <c r="I31">
+        <f t="shared" si="3"/>
+        <v>4.4580000000000055</v>
+      </c>
+      <c r="J31">
+        <f t="shared" si="4"/>
+        <v>19.873764000000048</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10">
       <c r="A32" s="1">
         <v>0</v>
       </c>
@@ -1861,8 +2226,20 @@
         <f t="shared" si="1"/>
         <v>9640.7461929957171</v>
       </c>
-    </row>
-    <row r="33" spans="1:5">
+      <c r="H32">
+        <f t="shared" si="2"/>
+        <v>19.989999999999998</v>
+      </c>
+      <c r="I32">
+        <f t="shared" si="3"/>
+        <v>-19.989999999999998</v>
+      </c>
+      <c r="J32">
+        <f t="shared" si="4"/>
+        <v>399.60009999999994</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10">
       <c r="A33" s="1">
         <v>25</v>
       </c>
@@ -1877,8 +2254,20 @@
         <f t="shared" si="1"/>
         <v>840.26365331317709</v>
       </c>
-    </row>
-    <row r="34" spans="1:5">
+      <c r="H33">
+        <f t="shared" si="2"/>
+        <v>105.31499999999998</v>
+      </c>
+      <c r="I33">
+        <f t="shared" si="3"/>
+        <v>-36.114999999999981</v>
+      </c>
+      <c r="J33">
+        <f t="shared" si="4"/>
+        <v>1304.2932249999985</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10">
       <c r="A34" s="1">
         <v>6</v>
       </c>
@@ -1893,8 +2282,20 @@
         <f t="shared" si="1"/>
         <v>6986.8369866465118</v>
       </c>
-    </row>
-    <row r="35" spans="1:5">
+      <c r="H34">
+        <f t="shared" si="2"/>
+        <v>40.467999999999996</v>
+      </c>
+      <c r="I34">
+        <f t="shared" si="3"/>
+        <v>-25.867999999999995</v>
+      </c>
+      <c r="J34">
+        <f t="shared" si="4"/>
+        <v>669.15342399999975</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10">
       <c r="A35" s="1">
         <v>5</v>
       </c>
@@ -1909,8 +2310,20 @@
         <f t="shared" si="1"/>
         <v>3350.9396850592098</v>
       </c>
-    </row>
-    <row r="36" spans="1:5">
+      <c r="H35">
+        <f t="shared" si="2"/>
+        <v>37.054999999999993</v>
+      </c>
+      <c r="I35">
+        <f t="shared" si="3"/>
+        <v>3.2450000000000045</v>
+      </c>
+      <c r="J35">
+        <f t="shared" si="4"/>
+        <v>10.53002500000003</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10">
       <c r="A36" s="1">
         <v>22</v>
       </c>
@@ -1925,8 +2338,20 @@
         <f t="shared" si="1"/>
         <v>4008.497780297304</v>
       </c>
-    </row>
-    <row r="37" spans="1:5">
+      <c r="H36">
+        <f t="shared" si="2"/>
+        <v>95.075999999999993</v>
+      </c>
+      <c r="I36">
+        <f t="shared" si="3"/>
+        <v>66.424000000000007</v>
+      </c>
+      <c r="J36">
+        <f t="shared" si="4"/>
+        <v>4412.1477760000007</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10">
       <c r="A37" s="1">
         <v>11</v>
       </c>
@@ -1941,8 +2366,20 @@
         <f t="shared" si="1"/>
         <v>1679.9588914084152</v>
       </c>
-    </row>
-    <row r="38" spans="1:5">
+      <c r="H37">
+        <f t="shared" si="2"/>
+        <v>57.533000000000001</v>
+      </c>
+      <c r="I37">
+        <f t="shared" si="3"/>
+        <v>-0.33299999999999841</v>
+      </c>
+      <c r="J37">
+        <f t="shared" si="4"/>
+        <v>0.11088899999999895</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10">
       <c r="A38" s="1">
         <v>61</v>
       </c>
@@ -1957,8 +2394,20 @@
         <f t="shared" si="1"/>
         <v>14259.392542202064</v>
       </c>
-    </row>
-    <row r="39" spans="1:5">
+      <c r="H38">
+        <f t="shared" si="2"/>
+        <v>228.18299999999999</v>
+      </c>
+      <c r="I38">
+        <f t="shared" si="3"/>
+        <v>-10.582999999999998</v>
+      </c>
+      <c r="J38">
+        <f t="shared" si="4"/>
+        <v>111.99988899999997</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10">
       <c r="A39" s="1">
         <v>12</v>
       </c>
@@ -1973,8 +2422,20 @@
         <f t="shared" si="1"/>
         <v>1606.9917485512724</v>
       </c>
-    </row>
-    <row r="40" spans="1:5">
+      <c r="H39">
+        <f t="shared" si="2"/>
+        <v>60.945999999999998</v>
+      </c>
+      <c r="I39">
+        <f t="shared" si="3"/>
+        <v>-2.8459999999999965</v>
+      </c>
+      <c r="J39">
+        <f t="shared" si="4"/>
+        <v>8.0997159999999795</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10">
       <c r="A40" s="1">
         <v>4</v>
       </c>
@@ -1989,8 +2450,20 @@
         <f t="shared" si="1"/>
         <v>7325.1861929957186</v>
       </c>
-    </row>
-    <row r="41" spans="1:5">
+      <c r="H40">
+        <f t="shared" si="2"/>
+        <v>33.641999999999996</v>
+      </c>
+      <c r="I40">
+        <f t="shared" si="3"/>
+        <v>-21.041999999999994</v>
+      </c>
+      <c r="J40">
+        <f t="shared" si="4"/>
+        <v>442.76576399999976</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10">
       <c r="A41" s="1">
         <v>16</v>
       </c>
@@ -2005,8 +2478,20 @@
         <f t="shared" si="1"/>
         <v>1488.9798437893678</v>
       </c>
-    </row>
-    <row r="42" spans="1:5">
+      <c r="H41">
+        <f t="shared" si="2"/>
+        <v>74.597999999999999</v>
+      </c>
+      <c r="I41">
+        <f t="shared" si="3"/>
+        <v>-14.997999999999998</v>
+      </c>
+      <c r="J41">
+        <f t="shared" si="4"/>
+        <v>224.94000399999993</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10">
       <c r="A42" s="1">
         <v>13</v>
       </c>
@@ -2021,8 +2506,20 @@
         <f t="shared" si="1"/>
         <v>68.679367598891361</v>
       </c>
-    </row>
-    <row r="43" spans="1:5">
+      <c r="H42">
+        <f t="shared" si="2"/>
+        <v>64.358999999999995</v>
+      </c>
+      <c r="I42">
+        <f t="shared" si="3"/>
+        <v>25.541000000000011</v>
+      </c>
+      <c r="J42">
+        <f t="shared" si="4"/>
+        <v>652.34268100000054</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10">
       <c r="A43" s="1">
         <v>60</v>
       </c>
@@ -2037,8 +2534,20 @@
         <f t="shared" si="1"/>
         <v>10860.286510456035</v>
       </c>
-    </row>
-    <row r="44" spans="1:5">
+      <c r="H43">
+        <f t="shared" si="2"/>
+        <v>224.77</v>
+      </c>
+      <c r="I43">
+        <f t="shared" si="3"/>
+        <v>-22.370000000000005</v>
+      </c>
+      <c r="J43">
+        <f t="shared" si="4"/>
+        <v>500.41690000000023</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10">
       <c r="A44" s="1">
         <v>41</v>
       </c>
@@ -2053,8 +2562,20 @@
         <f t="shared" si="1"/>
         <v>6907.720637440163</v>
       </c>
-    </row>
-    <row r="45" spans="1:5">
+      <c r="H44">
+        <f t="shared" si="2"/>
+        <v>159.923</v>
+      </c>
+      <c r="I44">
+        <f t="shared" si="3"/>
+        <v>21.37700000000001</v>
+      </c>
+      <c r="J44">
+        <f t="shared" si="4"/>
+        <v>456.97612900000041</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10">
       <c r="A45" s="1">
         <v>37</v>
       </c>
@@ -2069,8 +2590,20 @@
         <f t="shared" si="1"/>
         <v>2982.5468279163529</v>
       </c>
-    </row>
-    <row r="46" spans="1:5">
+      <c r="H45">
+        <f t="shared" si="2"/>
+        <v>146.27099999999999</v>
+      </c>
+      <c r="I45">
+        <f t="shared" si="3"/>
+        <v>6.5290000000000248</v>
+      </c>
+      <c r="J45">
+        <f t="shared" si="4"/>
+        <v>42.627841000000323</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10">
       <c r="A46" s="1">
         <v>55</v>
       </c>
@@ -2085,8 +2618,20 @@
         <f t="shared" si="1"/>
         <v>4174.8007961703215</v>
       </c>
-    </row>
-    <row r="47" spans="1:5">
+      <c r="H46">
+        <f t="shared" si="2"/>
+        <v>207.70500000000001</v>
+      </c>
+      <c r="I46">
+        <f t="shared" si="3"/>
+        <v>-44.905000000000001</v>
+      </c>
+      <c r="J46">
+        <f t="shared" si="4"/>
+        <v>2016.4590250000001</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10">
       <c r="A47" s="1">
         <v>41</v>
       </c>
@@ -2101,8 +2646,20 @@
         <f t="shared" si="1"/>
         <v>614.41031997984362</v>
       </c>
-    </row>
-    <row r="48" spans="1:5">
+      <c r="H47">
+        <f t="shared" si="2"/>
+        <v>159.923</v>
+      </c>
+      <c r="I47">
+        <f t="shared" si="3"/>
+        <v>-86.522999999999996</v>
+      </c>
+      <c r="J47">
+        <f t="shared" si="4"/>
+        <v>7486.2295289999993</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10">
       <c r="A48" s="1">
         <v>11</v>
       </c>
@@ -2117,8 +2674,20 @@
         <f t="shared" si="1"/>
         <v>5911.6571453766701</v>
       </c>
-    </row>
-    <row r="49" spans="1:5">
+      <c r="H48">
+        <f t="shared" si="2"/>
+        <v>57.533000000000001</v>
+      </c>
+      <c r="I48">
+        <f t="shared" si="3"/>
+        <v>-36.233000000000004</v>
+      </c>
+      <c r="J48">
+        <f t="shared" si="4"/>
+        <v>1312.8302890000002</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10">
       <c r="A49" s="1">
         <v>27</v>
       </c>
@@ -2133,8 +2702,20 @@
         <f t="shared" si="1"/>
         <v>31.217939027462933</v>
       </c>
-    </row>
-    <row r="50" spans="1:5">
+      <c r="H49">
+        <f t="shared" si="2"/>
+        <v>112.14099999999999</v>
+      </c>
+      <c r="I49">
+        <f t="shared" si="3"/>
+        <v>-19.540999999999997</v>
+      </c>
+      <c r="J49">
+        <f t="shared" si="4"/>
+        <v>381.85068099999989</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10">
       <c r="A50" s="1">
         <v>8</v>
       </c>
@@ -2149,8 +2730,20 @@
         <f t="shared" si="1"/>
         <v>487.84889140841562</v>
       </c>
-    </row>
-    <row r="51" spans="1:5">
+      <c r="H50">
+        <f t="shared" si="2"/>
+        <v>47.293999999999997</v>
+      </c>
+      <c r="I50">
+        <f t="shared" si="3"/>
+        <v>28.805999999999997</v>
+      </c>
+      <c r="J50">
+        <f t="shared" si="4"/>
+        <v>829.78563599999984</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10">
       <c r="A51" s="1">
         <v>3</v>
       </c>
@@ -2165,8 +2758,20 @@
         <f t="shared" si="1"/>
         <v>3397.4095263290505</v>
       </c>
-    </row>
-    <row r="52" spans="1:5">
+      <c r="H51">
+        <f t="shared" si="2"/>
+        <v>30.228999999999999</v>
+      </c>
+      <c r="I51">
+        <f t="shared" si="3"/>
+        <v>9.6709999999999994</v>
+      </c>
+      <c r="J51">
+        <f t="shared" si="4"/>
+        <v>93.528240999999994</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10">
       <c r="A52" s="1">
         <v>17</v>
       </c>
@@ -2181,8 +2786,20 @@
         <f t="shared" si="1"/>
         <v>1928.325081884605</v>
       </c>
-    </row>
-    <row r="53" spans="1:5">
+      <c r="H52">
+        <f t="shared" si="2"/>
+        <v>78.010999999999996</v>
+      </c>
+      <c r="I52">
+        <f t="shared" si="3"/>
+        <v>64.088999999999999</v>
+      </c>
+      <c r="J52">
+        <f t="shared" si="4"/>
+        <v>4107.3999210000002</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10">
       <c r="A53" s="1">
         <v>13</v>
       </c>
@@ -2197,8 +2814,20 @@
         <f t="shared" si="1"/>
         <v>26.908097757621597</v>
       </c>
-    </row>
-    <row r="54" spans="1:5">
+      <c r="H53">
+        <f t="shared" si="2"/>
+        <v>64.358999999999995</v>
+      </c>
+      <c r="I53">
+        <f t="shared" si="3"/>
+        <v>28.641000000000005</v>
+      </c>
+      <c r="J53">
+        <f t="shared" si="4"/>
+        <v>820.30688100000032</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10">
       <c r="A54" s="1">
         <v>13</v>
       </c>
@@ -2213,8 +2842,20 @@
         <f t="shared" si="1"/>
         <v>4394.006351725875</v>
       </c>
-    </row>
-    <row r="55" spans="1:5">
+      <c r="H54">
+        <f t="shared" si="2"/>
+        <v>64.358999999999995</v>
+      </c>
+      <c r="I54">
+        <f t="shared" si="3"/>
+        <v>-32.458999999999996</v>
+      </c>
+      <c r="J54">
+        <f t="shared" si="4"/>
+        <v>1053.5866809999998</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10">
       <c r="A55" s="1">
         <v>15</v>
       </c>
@@ -2229,8 +2870,20 @@
         <f t="shared" si="1"/>
         <v>4367.5314310909562</v>
       </c>
-    </row>
-    <row r="56" spans="1:5">
+      <c r="H55">
+        <f t="shared" si="2"/>
+        <v>71.185000000000002</v>
+      </c>
+      <c r="I55">
+        <f t="shared" si="3"/>
+        <v>-39.085000000000001</v>
+      </c>
+      <c r="J55">
+        <f t="shared" si="4"/>
+        <v>1527.6372250000002</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10">
       <c r="A56" s="1">
         <v>8</v>
       </c>
@@ -2245,8 +2898,20 @@
         <f t="shared" si="1"/>
         <v>1813.6782564877803</v>
       </c>
-    </row>
-    <row r="57" spans="1:5">
+      <c r="H56">
+        <f t="shared" si="2"/>
+        <v>47.293999999999997</v>
+      </c>
+      <c r="I56">
+        <f t="shared" si="3"/>
+        <v>8.3060000000000045</v>
+      </c>
+      <c r="J56">
+        <f t="shared" si="4"/>
+        <v>68.989636000000075</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10">
       <c r="A57" s="1">
         <v>29</v>
       </c>
@@ -2261,8 +2926,20 @@
         <f t="shared" si="1"/>
         <v>1232.9015898211142</v>
       </c>
-    </row>
-    <row r="58" spans="1:5">
+      <c r="H57">
+        <f t="shared" si="2"/>
+        <v>118.96699999999998</v>
+      </c>
+      <c r="I57">
+        <f t="shared" si="3"/>
+        <v>14.333000000000027</v>
+      </c>
+      <c r="J57">
+        <f t="shared" si="4"/>
+        <v>205.43488900000077</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10">
       <c r="A58" s="1">
         <v>30</v>
       </c>
@@ -2277,8 +2954,20 @@
         <f t="shared" si="1"/>
         <v>9276.1358755353995</v>
       </c>
-    </row>
-    <row r="59" spans="1:5">
+      <c r="H58">
+        <f t="shared" si="2"/>
+        <v>122.38</v>
+      </c>
+      <c r="I58">
+        <f t="shared" si="3"/>
+        <v>72.12</v>
+      </c>
+      <c r="J58">
+        <f t="shared" si="4"/>
+        <v>5201.2944000000007</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10">
       <c r="A59" s="1">
         <v>24</v>
       </c>
@@ -2293,8 +2982,20 @@
         <f t="shared" si="1"/>
         <v>1577.0984152179392</v>
       </c>
-    </row>
-    <row r="60" spans="1:5">
+      <c r="H59">
+        <f t="shared" si="2"/>
+        <v>101.90199999999999</v>
+      </c>
+      <c r="I59">
+        <f t="shared" si="3"/>
+        <v>35.998000000000019</v>
+      </c>
+      <c r="J59">
+        <f t="shared" si="4"/>
+        <v>1295.8560040000013</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10">
       <c r="A60" s="1">
         <v>9</v>
       </c>
@@ -2309,8 +3010,20 @@
         <f t="shared" si="1"/>
         <v>116.36587553539928</v>
       </c>
-    </row>
-    <row r="61" spans="1:5">
+      <c r="H60">
+        <f t="shared" si="2"/>
+        <v>50.706999999999994</v>
+      </c>
+      <c r="I60">
+        <f t="shared" si="3"/>
+        <v>36.693000000000012</v>
+      </c>
+      <c r="J60">
+        <f t="shared" si="4"/>
+        <v>1346.3762490000008</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10">
       <c r="A61" s="1">
         <v>31</v>
       </c>
@@ -2325,8 +3038,20 @@
         <f t="shared" si="1"/>
         <v>12457.394446963972</v>
       </c>
-    </row>
-    <row r="62" spans="1:5">
+      <c r="H61">
+        <f t="shared" si="2"/>
+        <v>125.79299999999999</v>
+      </c>
+      <c r="I61">
+        <f t="shared" si="3"/>
+        <v>84.007000000000019</v>
+      </c>
+      <c r="J61">
+        <f t="shared" si="4"/>
+        <v>7057.1760490000033</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10">
       <c r="A62" s="1">
         <v>14</v>
       </c>
@@ -2341,8 +3066,20 @@
         <f t="shared" si="1"/>
         <v>7.2215898211136462</v>
       </c>
-    </row>
-    <row r="63" spans="1:5">
+      <c r="H62">
+        <f t="shared" si="2"/>
+        <v>67.771999999999991</v>
+      </c>
+      <c r="I62">
+        <f t="shared" si="3"/>
+        <v>27.728000000000009</v>
+      </c>
+      <c r="J62">
+        <f t="shared" si="4"/>
+        <v>768.84198400000048</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10">
       <c r="A63" s="1">
         <v>53</v>
       </c>
@@ -2357,8 +3094,20 @@
         <f t="shared" si="1"/>
         <v>21436.678256487779</v>
       </c>
-    </row>
-    <row r="64" spans="1:5">
+      <c r="H63">
+        <f t="shared" si="2"/>
+        <v>200.87899999999999</v>
+      </c>
+      <c r="I63">
+        <f t="shared" si="3"/>
+        <v>43.721000000000004</v>
+      </c>
+      <c r="J63">
+        <f t="shared" si="4"/>
+        <v>1911.5258410000004</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10">
       <c r="A64" s="1">
         <v>26</v>
       </c>
@@ -2372,6 +3121,18 @@
       <c r="E64">
         <f t="shared" si="1"/>
         <v>7976.7580977576208</v>
+      </c>
+      <c r="H64">
+        <f t="shared" si="2"/>
+        <v>108.72799999999999</v>
+      </c>
+      <c r="I64">
+        <f t="shared" si="3"/>
+        <v>78.772000000000006</v>
+      </c>
+      <c r="J64">
+        <f t="shared" si="4"/>
+        <v>6205.0279840000012</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added code to calculate std deviation for population and sample
</commit_message>
<xml_diff>
--- a/Motor_Insurance_Regression/ClaimsVsPayment.xlsx
+++ b/Motor_Insurance_Regression/ClaimsVsPayment.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
   <si>
     <t>Xi</t>
   </si>
@@ -106,6 +106,9 @@
   </si>
   <si>
     <t>sse</t>
+  </si>
+  <si>
+    <t>stdev</t>
   </si>
 </sst>
 </file>
@@ -1311,7 +1314,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K64"/>
+  <dimension ref="A1:L64"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.28515625" bestFit="1" customWidth="1"/>
@@ -1324,7 +1327,7 @@
     <col min="9" max="9" width="13.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
         <v>26</v>
       </c>
@@ -1358,8 +1361,11 @@
       <c r="K1" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="2" spans="1:11">
+      <c r="L1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
       <c r="A2" s="1">
         <v>108</v>
       </c>
@@ -1398,8 +1404,12 @@
         <f>SUM(J2:J64)</f>
         <v>78796.798828999992</v>
       </c>
-    </row>
-    <row r="3" spans="1:11">
+      <c r="L2">
+        <f>STDEVP(B2:B64)</f>
+        <v>86.631704471877399</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
       <c r="A3" s="1">
         <v>19</v>
       </c>
@@ -1427,7 +1437,7 @@
         <v>1492.8177689999989</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:12">
       <c r="A4" s="1">
         <v>13</v>
       </c>
@@ -1455,7 +1465,7 @@
         <v>2367.698280999999</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:12">
       <c r="A5" s="1">
         <v>124</v>
       </c>
@@ -1483,7 +1493,7 @@
         <v>441.08400400000039</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:12">
       <c r="A6" s="1">
         <v>40</v>
       </c>
@@ -1511,7 +1521,7 @@
         <v>1377.1520999999989</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:12">
       <c r="A7" s="1">
         <v>57</v>
       </c>
@@ -1539,7 +1549,7 @@
         <v>1903.6641609999999</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:12">
       <c r="A8" s="1">
         <v>23</v>
       </c>
@@ -1567,7 +1577,7 @@
         <v>1729.6449209999994</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:12">
       <c r="A9" s="1">
         <v>14</v>
       </c>
@@ -1595,7 +1605,7 @@
         <v>94.633984000000169</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:12">
       <c r="A10" s="1">
         <v>45</v>
       </c>
@@ -1623,7 +1633,7 @@
         <v>1634.1806250000009</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:12">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -1651,7 +1661,7 @@
         <v>124.99240000000015</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:12">
       <c r="A12" s="1">
         <v>5</v>
       </c>
@@ -1679,7 +1689,7 @@
         <v>260.9840249999998</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:12">
       <c r="A13" s="1">
         <v>48</v>
       </c>
@@ -1707,7 +1717,7 @@
         <v>4132.6897960000006</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:12">
       <c r="A14" s="1">
         <v>11</v>
       </c>
@@ -1735,7 +1745,7 @@
         <v>1158.245089</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:12">
       <c r="A15" s="1">
         <v>23</v>
       </c>
@@ -1763,7 +1773,7 @@
         <v>3467.9143209999988</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:12">
       <c r="A16" s="1">
         <v>7</v>
       </c>

</xml_diff>

<commit_message>
Added code to calculate karl pearson coeff of correlation
</commit_message>
<xml_diff>
--- a/Motor_Insurance_Regression/ClaimsVsPayment.xlsx
+++ b/Motor_Insurance_Regression/ClaimsVsPayment.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="34">
   <si>
     <t>Xi</t>
   </si>
@@ -110,13 +110,30 @@
   <si>
     <t>stdev</t>
   </si>
+  <si>
+    <t>std</t>
+  </si>
+  <si>
+    <t>covariance</t>
+  </si>
+  <si>
+    <t>Correlation</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -132,7 +149,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -140,14 +157,39 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -593,23 +635,23 @@
             </c:numRef>
           </c:yVal>
         </c:ser>
-        <c:axId val="68107648"/>
-        <c:axId val="68121728"/>
+        <c:axId val="74018176"/>
+        <c:axId val="74032256"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="68107648"/>
+        <c:axId val="74018176"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="b"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="68121728"/>
+        <c:crossAx val="74032256"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="68121728"/>
+        <c:axId val="74032256"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -617,7 +659,7 @@
         <c:majorGridlines/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="68107648"/>
+        <c:crossAx val="74018176"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -630,7 +672,7 @@
   </c:chart>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75000000000000089" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000089" header="0.30000000000000032" footer="0.30000000000000032"/>
+    <c:pageMargins b="0.750000000000001" l="0.70000000000000062" r="0.70000000000000062" t="0.750000000000001" header="0.30000000000000032" footer="0.30000000000000032"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -771,23 +813,23 @@
             </c:numRef>
           </c:yVal>
         </c:ser>
-        <c:axId val="80653696"/>
-        <c:axId val="80655488"/>
+        <c:axId val="74116480"/>
+        <c:axId val="74118272"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="80653696"/>
+        <c:axId val="74116480"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="b"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="80655488"/>
+        <c:crossAx val="74118272"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="80655488"/>
+        <c:axId val="74118272"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -795,7 +837,7 @@
         <c:majorGridlines/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="80653696"/>
+        <c:crossAx val="74116480"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -808,7 +850,7 @@
   </c:chart>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75000000000000089" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000089" header="0.30000000000000032" footer="0.30000000000000032"/>
+    <c:pageMargins b="0.750000000000001" l="0.70000000000000062" r="0.70000000000000062" t="0.750000000000001" header="0.30000000000000032" footer="0.30000000000000032"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -818,9 +860,7 @@
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:chart>
-    <c:title>
-      <c:layout/>
-    </c:title>
+    <c:title/>
     <c:plotArea>
       <c:layout/>
       <c:scatterChart>
@@ -881,23 +921,23 @@
             </c:numRef>
           </c:yVal>
         </c:ser>
-        <c:axId val="80667776"/>
-        <c:axId val="80669312"/>
+        <c:axId val="74204288"/>
+        <c:axId val="74205824"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="80667776"/>
+        <c:axId val="74204288"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="b"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="80669312"/>
+        <c:crossAx val="74205824"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="80669312"/>
+        <c:axId val="74205824"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -905,20 +945,19 @@
         <c:majorGridlines/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="80667776"/>
+        <c:crossAx val="74204288"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
-      <c:layout/>
     </c:legend>
     <c:plotVisOnly val="1"/>
   </c:chart>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75000000000000056" l="0.70000000000000051" r="0.70000000000000051" t="0.75000000000000056" header="0.30000000000000027" footer="0.30000000000000027"/>
+    <c:pageMargins b="0.75000000000000078" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000078" header="0.30000000000000032" footer="0.30000000000000032"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -1314,7 +1353,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L64"/>
+  <dimension ref="A1:R64"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.28515625" bestFit="1" customWidth="1"/>
@@ -1325,9 +1364,11 @@
     <col min="7" max="7" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:18" ht="15.75" thickBot="1">
       <c r="A1" s="1" t="s">
         <v>26</v>
       </c>
@@ -1364,8 +1405,14 @@
       <c r="L1" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="2" spans="1:12">
+      <c r="M1" t="s">
+        <v>32</v>
+      </c>
+      <c r="P1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18">
       <c r="A2" s="1">
         <v>108</v>
       </c>
@@ -1408,8 +1455,22 @@
         <f>STDEVP(B2:B64)</f>
         <v>86.631704471877399</v>
       </c>
-    </row>
-    <row r="3" spans="1:12">
+      <c r="M2" s="4"/>
+      <c r="N2" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="O2" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="P2" s="4"/>
+      <c r="Q2" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="R2" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18">
       <c r="A3" s="1">
         <v>19</v>
       </c>
@@ -1436,8 +1497,23 @@
         <f t="shared" ref="J3:J64" si="4">I3*I3</f>
         <v>1492.8177689999989</v>
       </c>
-    </row>
-    <row r="4" spans="1:12">
+      <c r="M3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N3" s="2">
+        <f>VARP(ClaimsVsPayment!$A$2:$A$64)</f>
+        <v>536.65759637188205</v>
+      </c>
+      <c r="O3" s="2"/>
+      <c r="P3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q3" s="2">
+        <v>1</v>
+      </c>
+      <c r="R3" s="2"/>
+    </row>
+    <row r="4" spans="1:18" ht="15.75" thickBot="1">
       <c r="A4" s="1">
         <v>13</v>
       </c>
@@ -1464,8 +1540,27 @@
         <f t="shared" si="4"/>
         <v>2367.698280999999</v>
       </c>
-    </row>
-    <row r="5" spans="1:12">
+      <c r="M4" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="N4" s="3">
+        <v>1832.0543461829182</v>
+      </c>
+      <c r="O4" s="3">
+        <f>VARP(ClaimsVsPayment!$B$2:$B$64)</f>
+        <v>7505.0522197027012</v>
+      </c>
+      <c r="P4" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q4" s="3">
+        <v>0.91287823502340715</v>
+      </c>
+      <c r="R4" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18">
       <c r="A5" s="1">
         <v>124</v>
       </c>
@@ -1493,7 +1588,7 @@
         <v>441.08400400000039</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="1:18">
       <c r="A6" s="1">
         <v>40</v>
       </c>
@@ -1521,7 +1616,7 @@
         <v>1377.1520999999989</v>
       </c>
     </row>
-    <row r="7" spans="1:12">
+    <row r="7" spans="1:18">
       <c r="A7" s="1">
         <v>57</v>
       </c>
@@ -1549,7 +1644,7 @@
         <v>1903.6641609999999</v>
       </c>
     </row>
-    <row r="8" spans="1:12">
+    <row r="8" spans="1:18">
       <c r="A8" s="1">
         <v>23</v>
       </c>
@@ -1577,7 +1672,7 @@
         <v>1729.6449209999994</v>
       </c>
     </row>
-    <row r="9" spans="1:12">
+    <row r="9" spans="1:18">
       <c r="A9" s="1">
         <v>14</v>
       </c>
@@ -1605,7 +1700,7 @@
         <v>94.633984000000169</v>
       </c>
     </row>
-    <row r="10" spans="1:12">
+    <row r="10" spans="1:18">
       <c r="A10" s="1">
         <v>45</v>
       </c>
@@ -1633,7 +1728,7 @@
         <v>1634.1806250000009</v>
       </c>
     </row>
-    <row r="11" spans="1:12">
+    <row r="11" spans="1:18">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -1661,7 +1756,7 @@
         <v>124.99240000000015</v>
       </c>
     </row>
-    <row r="12" spans="1:12">
+    <row r="12" spans="1:18">
       <c r="A12" s="1">
         <v>5</v>
       </c>
@@ -1689,7 +1784,7 @@
         <v>260.9840249999998</v>
       </c>
     </row>
-    <row r="13" spans="1:12">
+    <row r="13" spans="1:18">
       <c r="A13" s="1">
         <v>48</v>
       </c>
@@ -1717,7 +1812,7 @@
         <v>4132.6897960000006</v>
       </c>
     </row>
-    <row r="14" spans="1:12">
+    <row r="14" spans="1:18">
       <c r="A14" s="1">
         <v>11</v>
       </c>
@@ -1745,7 +1840,7 @@
         <v>1158.245089</v>
       </c>
     </row>
-    <row r="15" spans="1:12">
+    <row r="15" spans="1:18">
       <c r="A15" s="1">
         <v>23</v>
       </c>
@@ -1773,7 +1868,7 @@
         <v>3467.9143209999988</v>
       </c>
     </row>
-    <row r="16" spans="1:12">
+    <row r="16" spans="1:18">
       <c r="A16" s="1">
         <v>7</v>
       </c>
@@ -3153,7 +3248,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="31.85546875" bestFit="1" customWidth="1"/>
@@ -3163,7 +3258,7 @@
     <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>15</v>
       </c>
@@ -3179,8 +3274,11 @@
       <c r="E1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="F1" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2" s="1">
         <v>108</v>
       </c>
@@ -3199,8 +3297,12 @@
         <f>B2-$C$2</f>
         <v>238.36666666666667</v>
       </c>
-    </row>
-    <row r="3" spans="1:5">
+      <c r="F2">
+        <f>STDEVP(B2:B13)</f>
+        <v>133.65457551298255</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3" s="1">
         <v>19</v>
       </c>
@@ -3217,7 +3319,7 @@
         <v>-107.93333333333332</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:6">
       <c r="A4" s="1">
         <v>13</v>
       </c>
@@ -3234,7 +3336,7 @@
         <v>-138.43333333333334</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:6">
       <c r="A5" s="1">
         <v>124</v>
       </c>
@@ -3251,7 +3353,7 @@
         <v>268.06666666666666</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:6">
       <c r="A6" s="1">
         <v>40</v>
       </c>
@@ -3268,7 +3370,7 @@
         <v>-34.73333333333332</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:6">
       <c r="A7" s="1">
         <v>57</v>
       </c>
@@ -3285,7 +3387,7 @@
         <v>16.76666666666668</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:6">
       <c r="A8" s="1">
         <v>23</v>
       </c>
@@ -3302,7 +3404,7 @@
         <v>-97.23333333333332</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:6">
       <c r="A9" s="1">
         <v>14</v>
       </c>
@@ -3319,7 +3421,7 @@
         <v>-76.633333333333326</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:6">
       <c r="A10" s="1">
         <v>45</v>
       </c>
@@ -3336,7 +3438,7 @@
         <v>59.866666666666674</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:6">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -3353,7 +3455,7 @@
         <v>-88.833333333333329</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:6">
       <c r="A12" s="1">
         <v>5</v>
       </c>
@@ -3370,7 +3472,7 @@
         <v>-133.23333333333332</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:6">
       <c r="A13" s="1">
         <v>48</v>
       </c>

</xml_diff>